<commit_message>
docs/completed- thesaurus- and- summaries- 1-10
</commit_message>
<xml_diff>
--- a/02-week/02-session/02-activity/Thesaurus.xlsx
+++ b/02-week/02-session/02-activity/Thesaurus.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\USER\OneDrive\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{56838547-D55F-46A3-AC3A-8A3460F21C1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D69153CA-2FC8-4A37-AF4D-F6D7BE22283F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11760" xr2:uid="{0B9C9D57-2DC8-48FF-9917-C6D5FE53AD36}"/>
   </bookViews>
@@ -130,12 +130,6 @@
     <t>"Programacion orientada a objetos"</t>
   </si>
   <si>
-    <t>http://www.scielo.org.bo/pdf/ran/v2n4/v2n4_a05.pdf</t>
-  </si>
-  <si>
-    <t>El patrón de diseño Modelo-Vista-Controlador (MVC) y su implementación en Java Swing</t>
-  </si>
-  <si>
     <t>"Calidad de Software"</t>
   </si>
   <si>
@@ -217,9 +211,6 @@
     <t>"moviles" y "TypeScript"</t>
   </si>
   <si>
-    <t>"MVC" y "java"</t>
-  </si>
-  <si>
     <t>Implementación de métodos ágiles para la simulación de casos de 
 uso y prototipado en el proceso de desarrollo de software</t>
   </si>
@@ -256,6 +247,15 @@
   </si>
   <si>
     <t>https://revistas.ucc.edu.co/index.php/in/article/view/1482</t>
+  </si>
+  <si>
+    <t xml:space="preserve">"MVC" </t>
+  </si>
+  <si>
+    <t xml:space="preserve">Patrón Modelo-Vista-Controlador. </t>
+  </si>
+  <si>
+    <t>https://d1wqtxts1xzle7.cloudfront.net/38870522/15-42-2-PB-libre.pdf?1443047540=&amp;response-content-disposition=inline%3B+filename%3DPatron_Modelo_Vista_Controlador.pdf&amp;Expires=1756059628&amp;Signature=G1iVGRjIxA2SmHnrUtIgGipgaXx1FE4fMs90hXU-RoguQmIS4FroyuoPwjcw2V2kyeCmaZyR6Wvoy3MhcjCLqYYz6tXUkKQseXmUf8OudBTzJC5taJEKT8QzIrnfn8Vlv~rXozm2UIOmjEU5HlVeRNzyMhzrhcDasHh-~HJvTKG8VEiXUoxgm35fI9oKJAnwLAPnRWy6~fVmNkURNAu7Sw6sS4st0wm8C1yYB5OxUw4Eb1U7LR3jXQkiFduj5NLwNVngo2zpclK57N97iopp-cceusd4GXoIoOlMesZPscm7pk3FjMTmg~IRjR4tLmQLj7Q8aItIXRBU2SFwF~2eXg__&amp;Key-Pair-Id=APKAJLOHF5GGSLRBV4ZA</t>
   </si>
 </sst>
 </file>
@@ -305,7 +305,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="4">
+  <fills count="6">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -321,6 +321,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="0"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -366,7 +378,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -389,6 +401,8 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="2" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -704,7 +718,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{70BBECF4-C1D4-40AB-9B71-1D546767BA8D}">
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:H21"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="2" max="2" width="19.5703125" customWidth="1"/>
@@ -715,7 +729,7 @@
     <col min="7" max="7" width="14.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="30" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -738,7 +752,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="2" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>1</v>
       </c>
@@ -761,7 +775,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A3" s="2">
         <v>2</v>
       </c>
@@ -784,7 +798,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A4" s="2">
         <v>3</v>
       </c>
@@ -795,19 +809,20 @@
         <v>2008</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="E4" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F4" s="5" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="G4" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="5" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H4" s="8"/>
+    </row>
+    <row r="5" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A5" s="2">
         <v>4</v>
       </c>
@@ -818,7 +833,7 @@
         <v>2017</v>
       </c>
       <c r="D5" s="4" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="E5" s="2" t="s">
         <v>8</v>
@@ -830,7 +845,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="6" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A6" s="2">
         <v>5</v>
       </c>
@@ -853,7 +868,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="7" spans="1:7" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:8" ht="89.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A7" s="2">
         <v>6</v>
       </c>
@@ -876,7 +891,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="8" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:8" ht="75" x14ac:dyDescent="0.25">
       <c r="A8" s="2">
         <v>7</v>
       </c>
@@ -899,12 +914,12 @@
         <v>7</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A9" s="2">
         <v>8</v>
       </c>
       <c r="B9" s="3" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="C9" s="2">
         <v>2021</v>
@@ -922,7 +937,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="10" spans="1:7" ht="60" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:8" ht="60" x14ac:dyDescent="0.25">
       <c r="A10" s="2">
         <v>9</v>
       </c>
@@ -933,151 +948,152 @@
         <v>2023</v>
       </c>
       <c r="D10" s="4" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E10" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F10" s="5" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="G10" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="11" spans="1:7" ht="75" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:8" ht="345" x14ac:dyDescent="0.25">
       <c r="A11" s="2">
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>57</v>
+        <v>67</v>
       </c>
       <c r="C11" s="2">
-        <v>2004</v>
+        <v>2012</v>
       </c>
       <c r="D11" s="4" t="s">
-        <v>31</v>
+        <v>69</v>
       </c>
       <c r="E11" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F11" s="5" t="s">
-        <v>32</v>
+        <v>68</v>
       </c>
       <c r="G11" s="2" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="12" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+      <c r="H11" s="9"/>
+    </row>
+    <row r="12" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A12" s="2">
         <v>11</v>
       </c>
       <c r="B12" s="3" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="C12" s="2">
         <v>2016</v>
       </c>
       <c r="D12" s="4" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="E12" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F12" s="5" t="s">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="G12" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="13" spans="1:7" ht="360" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:8" ht="360" x14ac:dyDescent="0.25">
       <c r="A13" s="2">
         <v>12</v>
       </c>
       <c r="B13" s="3" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="C13" s="2">
         <v>2019</v>
       </c>
       <c r="D13" s="4" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="E13" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F13" s="5" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="G13" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="14" spans="1:7" ht="45" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:8" ht="45" x14ac:dyDescent="0.25">
       <c r="A14" s="2">
         <v>13</v>
       </c>
       <c r="B14" s="3" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="C14" s="2">
         <v>2020</v>
       </c>
       <c r="D14" s="4" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E14" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F14" s="5" t="s">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="G14" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="15" spans="1:7" ht="90" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:8" ht="90" x14ac:dyDescent="0.25">
       <c r="A15" s="2">
         <v>14</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="C15" s="2">
         <v>2024</v>
       </c>
       <c r="D15" s="4" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F15" s="5" t="s">
         <v>41</v>
       </c>
-      <c r="E15" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="F15" s="5" t="s">
-        <v>43</v>
-      </c>
       <c r="G15" s="2" t="s">
         <v>7</v>
       </c>
     </row>
-    <row r="16" spans="1:7" ht="150" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:8" ht="150" x14ac:dyDescent="0.25">
       <c r="A16" s="2">
         <v>15</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="C16" s="2">
         <v>2014</v>
       </c>
       <c r="D16" s="4" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
       <c r="E16" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F16" s="5" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="G16" s="2" t="s">
         <v>7</v>
@@ -1088,19 +1104,19 @@
         <v>16</v>
       </c>
       <c r="B17" s="3" t="s">
-        <v>49</v>
+        <v>47</v>
       </c>
       <c r="C17" s="2">
         <v>2020</v>
       </c>
       <c r="D17" s="4" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="E17" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F17" s="5" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
       <c r="G17" s="2" t="s">
         <v>7</v>
@@ -1111,19 +1127,19 @@
         <v>17</v>
       </c>
       <c r="B18" s="3" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="C18" s="2">
         <v>2015</v>
       </c>
       <c r="D18" s="4" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="E18" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F18" s="5" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="G18" s="2" t="s">
         <v>7</v>
@@ -1134,19 +1150,19 @@
         <v>18</v>
       </c>
       <c r="B19" s="3" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="C19" s="2">
         <v>2019</v>
       </c>
       <c r="D19" s="4" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="E19" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="G19" s="2" t="s">
         <v>7</v>
@@ -1157,19 +1173,19 @@
         <v>19</v>
       </c>
       <c r="B20" s="3" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="C20" s="2">
         <v>2013</v>
       </c>
       <c r="D20" s="4" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E20" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F20" s="5" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="G20" s="2" t="s">
         <v>7</v>
@@ -1180,19 +1196,19 @@
         <v>20</v>
       </c>
       <c r="B21" s="3" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="C21" s="2">
         <v>2024</v>
       </c>
       <c r="D21" s="4" t="s">
-        <v>63</v>
+        <v>60</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>8</v>
       </c>
       <c r="F21" s="5" t="s">
-        <v>64</v>
+        <v>61</v>
       </c>
       <c r="G21" s="2" t="s">
         <v>7</v>
@@ -1210,17 +1226,17 @@
     <hyperlink ref="D8" r:id="rId7" xr:uid="{72FF45EA-B60E-4350-A668-F643CA3A2142}"/>
     <hyperlink ref="D9" r:id="rId8" xr:uid="{ADF7A2A5-0193-4ACF-8B17-A0AC60B0C3C7}"/>
     <hyperlink ref="D10" r:id="rId9" xr:uid="{96DAC802-CC1C-442C-9639-2A1A191B50F5}"/>
-    <hyperlink ref="D11" r:id="rId10" xr:uid="{F9FBC1A2-1F1D-411D-BA00-7CCB451D6017}"/>
-    <hyperlink ref="D12" r:id="rId11" xr:uid="{B3196F29-A027-48DE-900D-E6F48C4E4A50}"/>
-    <hyperlink ref="D13" r:id="rId12" display="https://d1wqtxts1xzle7.cloudfront.net/98684258/pdf-libre.pdf?1676425601=&amp;response-content-disposition=inline%3B+filename%3DCatalogo_de_refactorizacion_de_codigo_fu.pdf&amp;Expires=1755875562&amp;Signature=ADH7Y-2-TuFv7yxwuSxwOwdePmV~Olz0zvqWbSFkrbsqXsBAOl0mfF5LItlg3Tlc6p9dpxBRrHe9TXOlK6x0Y5PzDJ2CsGtZTiQU7rgcc0~Bp7dA0cVmfMvqXcf5~AR5ZWIQQg41lEoN5LG2UlLDS-uJrGIbYt9zPvzdcP2mgsx0NmIhfM3nlWBPC8tc4pvz5TZmq5Hs9~-TwaCcRqCPu6x~VTwev2excyGYeDeceQGaL~PNTPvUaOkzIo2fPGB~y~U8boDbVS6QS9VaBNNyvTidN4rCbydEGdSRuwhst2mJ5QxQpzM48PyPU1aKD~9GaPkQaUEp6JzftXPfVfKcPw__&amp;Key-Pair-Id=APKAJLOHF5GGSLRBV4ZA" xr:uid="{A34A9D79-D8F4-4C8D-819B-FA58EE7F19DB}"/>
-    <hyperlink ref="D14" r:id="rId13" xr:uid="{FA51C115-40EA-4898-8721-B34D4574F1AA}"/>
-    <hyperlink ref="D15" r:id="rId14" xr:uid="{33416928-041B-462F-92FC-EFEA8B953631}"/>
-    <hyperlink ref="D16" r:id="rId15" xr:uid="{959DFC59-512A-4E27-B201-90C6C79B078A}"/>
-    <hyperlink ref="D17" r:id="rId16" xr:uid="{9D49A71B-39AF-4828-8429-A143E424FACF}"/>
-    <hyperlink ref="D18" r:id="rId17" xr:uid="{2F99A99A-D855-4B8E-BC3A-0B6CE49BDD78}"/>
-    <hyperlink ref="D19" r:id="rId18" xr:uid="{66EA81A0-3D10-4D88-9D6D-F3F0F53A19CC}"/>
-    <hyperlink ref="D20" r:id="rId19" xr:uid="{CD95FE34-E000-4786-B637-207D51E630E6}"/>
-    <hyperlink ref="D21" r:id="rId20" xr:uid="{917B1482-06BC-48B1-B4F3-B808291EDD04}"/>
+    <hyperlink ref="D12" r:id="rId10" xr:uid="{B3196F29-A027-48DE-900D-E6F48C4E4A50}"/>
+    <hyperlink ref="D13" r:id="rId11" display="https://d1wqtxts1xzle7.cloudfront.net/98684258/pdf-libre.pdf?1676425601=&amp;response-content-disposition=inline%3B+filename%3DCatalogo_de_refactorizacion_de_codigo_fu.pdf&amp;Expires=1755875562&amp;Signature=ADH7Y-2-TuFv7yxwuSxwOwdePmV~Olz0zvqWbSFkrbsqXsBAOl0mfF5LItlg3Tlc6p9dpxBRrHe9TXOlK6x0Y5PzDJ2CsGtZTiQU7rgcc0~Bp7dA0cVmfMvqXcf5~AR5ZWIQQg41lEoN5LG2UlLDS-uJrGIbYt9zPvzdcP2mgsx0NmIhfM3nlWBPC8tc4pvz5TZmq5Hs9~-TwaCcRqCPu6x~VTwev2excyGYeDeceQGaL~PNTPvUaOkzIo2fPGB~y~U8boDbVS6QS9VaBNNyvTidN4rCbydEGdSRuwhst2mJ5QxQpzM48PyPU1aKD~9GaPkQaUEp6JzftXPfVfKcPw__&amp;Key-Pair-Id=APKAJLOHF5GGSLRBV4ZA" xr:uid="{A34A9D79-D8F4-4C8D-819B-FA58EE7F19DB}"/>
+    <hyperlink ref="D14" r:id="rId12" xr:uid="{FA51C115-40EA-4898-8721-B34D4574F1AA}"/>
+    <hyperlink ref="D15" r:id="rId13" xr:uid="{33416928-041B-462F-92FC-EFEA8B953631}"/>
+    <hyperlink ref="D16" r:id="rId14" xr:uid="{959DFC59-512A-4E27-B201-90C6C79B078A}"/>
+    <hyperlink ref="D17" r:id="rId15" xr:uid="{9D49A71B-39AF-4828-8429-A143E424FACF}"/>
+    <hyperlink ref="D18" r:id="rId16" xr:uid="{2F99A99A-D855-4B8E-BC3A-0B6CE49BDD78}"/>
+    <hyperlink ref="D19" r:id="rId17" xr:uid="{66EA81A0-3D10-4D88-9D6D-F3F0F53A19CC}"/>
+    <hyperlink ref="D20" r:id="rId18" xr:uid="{CD95FE34-E000-4786-B637-207D51E630E6}"/>
+    <hyperlink ref="D21" r:id="rId19" xr:uid="{917B1482-06BC-48B1-B4F3-B808291EDD04}"/>
+    <hyperlink ref="D11" r:id="rId20" display="https://d1wqtxts1xzle7.cloudfront.net/38870522/15-42-2-PB-libre.pdf?1443047540=&amp;response-content-disposition=inline%3B+filename%3DPatron_Modelo_Vista_Controlador.pdf&amp;Expires=1756059628&amp;Signature=G1iVGRjIxA2SmHnrUtIgGipgaXx1FE4fMs90hXU-RoguQmIS4FroyuoPwjcw2V2kyeCmaZyR6Wvoy3MhcjCLqYYz6tXUkKQseXmUf8OudBTzJC5taJEKT8QzIrnfn8Vlv~rXozm2UIOmjEU5HlVeRNzyMhzrhcDasHh-~HJvTKG8VEiXUoxgm35fI9oKJAnwLAPnRWy6~fVmNkURNAu7Sw6sS4st0wm8C1yYB5OxUw4Eb1U7LR3jXQkiFduj5NLwNVngo2zpclK57N97iopp-cceusd4GXoIoOlMesZPscm7pk3FjMTmg~IRjR4tLmQLj7Q8aItIXRBU2SFwF~2eXg__&amp;Key-Pair-Id=APKAJLOHF5GGSLRBV4ZA" xr:uid="{C9E962F7-2AE8-41A0-BE95-66E29E8D1142}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId21"/>

</xml_diff>